<commit_message>
test(v1.0): consolidate shared seed data across all TC modules [AI]
Add Project_rule §10.3 to require one shared seed block per module
instead of repeating "nhờ dev/QA seed" per TC, and prefer creating
order states via real UI flow over DB seeding. Revise all 11 TC
fragments accordingly (~85% of 219 TC now self-servable); re-sync
TC-MASTER for ACT only, other modules flagged as pending full
consolidate due to pre-existing xlsx/fragment drift.

Refs: N/A
</commit_message>
<xml_diff>
--- a/03_test-cases/TC-MASTER-LATEST.xlsx
+++ b/03_test-cases/TC-MASTER-LATEST.xlsx
@@ -513,7 +513,6 @@
           <t>TC-MASTER — foxeco-v2</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -645,7 +644,6 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -7582,7 +7580,7 @@
       <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Tài khoản SSO CBNV FPT còn hiệu lực trên STG.
-- Host app FoxPro (`vn.fpt.ftel.sop.stg`) đã cài trên thiết bị Android.</t>
+- Host app FoxPro (`vn.fpt.ftel.sop.stg`) đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
@@ -8828,24 +8826,24 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG.</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment).
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed cho tài khoản đủ 4 đơn đang hoạt động ở các trạng thái "Chờ ghép", "Đã ghép", "Đang giao", "Đã giao", cùng 1 đơn "Hoàn thành" và 1 đơn "Hết hạn". (setup)
-2. Đăng nhập FoxEco và nhấn tab "Hoạt động".
-3. Check badge trạng thái của từng card trong tab "Đang diễn ra".</t>
+          <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
+2. Check badge trạng thái của từng card trong tab "Đang diễn ra".</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>3. Mọi card trong danh sách có badge thuộc nhóm "Chờ ghép", "Đã ghép", "Đang giao", "Đã giao"; KHÔNG có card nào badge "Hoàn thành" hoặc "Hết hạn".</t>
+          <t>2. Mọi card trong danh sách có badge thuộc nhóm "Chờ ghép", "Đã ghép", "Đang giao", "Đã giao"; KHÔNG có card nào badge "Hoàn thành" hoặc "Hết hạn".</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>4 đơn đang hoạt động + 1 đơn "Hoàn thành" + 1 đơn "Hết hạn" (test_data_catalog §ACT)</t>
+          <t>4 đơn đang hoạt động + 1 đơn "Hoàn thành" + 1 đơn "Hết hạn" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr"/>
@@ -8904,25 +8902,25 @@
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG.</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment).
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed cho tài khoản 1 đơn "Hoàn thành", 1 đơn "Hết hạn" và 1 đơn "Đang giao". (setup)
-2. Đăng nhập FoxEco và nhấn tab "Hoạt động".
-3. Nhấn tab con "Đã hoàn thành".
-4. Check badge trạng thái của từng card trong danh sách.</t>
+          <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
+2. Nhấn tab con "Đã hoàn thành". (setup)
+3. Check badge trạng thái của từng card trong danh sách.</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t>4. Danh sách có card badge "Hoàn thành" và card badge "Hết hạn"; KHÔNG có card nào badge "Chờ ghép", "Đã ghép", "Đang giao" hay "Đã giao".</t>
+          <t>3. Danh sách có card badge "Hoàn thành" và card badge "Hết hạn"; KHÔNG có card nào badge "Chờ ghép", "Đã ghép", "Đang giao" hay "Đã giao".</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>1 đơn "Hoàn thành" + 1 đơn "Hết hạn" + 1 đơn "Đang giao" (test_data_catalog §ACT)</t>
+          <t>1 đơn "Hoàn thành" + 1 đơn "Hết hạn" + 1 đơn "Đang giao" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr"/>
@@ -8981,24 +8979,24 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG có ≥1 đơn đang hoạt động.</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment).
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed cho tài khoản 1 đơn ở trạng thái "Đang giao". (setup)
-2. Đăng nhập FoxEco và nhấn tab "Hoạt động".
-3. Check lần lượt các trường trên card đơn.</t>
+          <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
+2. Check lần lượt các trường trên card đơn "Đang giao".</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>3. Card hiển thị đủ 5 trường: icon trạng thái, tên tin, tuyến đường dạng "Từ → Đến", ngày, badge trạng thái.</t>
+          <t>2. Card hiển thị đủ 5 trường: icon trạng thái, tên tin, tuyến đường dạng "Từ → Đến", ngày, badge trạng thái.</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>1 đơn "Đang giao" (test_data_catalog §ACT)</t>
+          <t>Đơn "Đang giao" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr"/>
@@ -9134,25 +9132,25 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG.</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment) — bất kỳ 2 đơn active nào trong bộ này đã khác tên tin/tuyến sẵn.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed cho tài khoản 2 đơn đang hoạt động khác nhau về tên tin và tuyến đường. (setup)
-2. Đăng nhập FoxEco và nhấn tab "Hoạt động".
-3. Ghi lại tên tin và tuyến đường của card thứ hai.
-4. Nhấn vào card thứ hai.</t>
+          <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
+2. Ghi lại tên tin và tuyến đường của card thứ hai.
+3. Nhấn vào card thứ hai.</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>4. Màn vừa mở hiển thị tên tin và tuyến đường trùng khớp thông tin đã ghi ở bước 3.</t>
+          <t>3. Màn vừa mở hiển thị tên tin và tuyến đường trùng khớp thông tin đã ghi ở bước 2.</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>2 đơn đang hoạt động khác nhau (test_data_catalog §ACT)</t>
+          <t>2 đơn đang hoạt động khác nhau của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr"/>
@@ -9211,26 +9209,26 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG có ≥1 đơn đang hoạt động và ≥1 đơn đã kết thúc.</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment).
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed cho tài khoản 1 đơn ở trạng thái "Đang giao" và 1 đơn ở trạng thái "Hoàn thành". (setup)
-2. Đăng nhập FoxEco và nhấn tab "Hoạt động".
-3. Nhấn tab con "Đã hoàn thành".
-4. Nhấn tab con "Đang diễn ra".</t>
+          <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
+2. Nhấn tab con "Đã hoàn thành".
+3. Nhấn tab con "Đang diễn ra".</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>3. Tab "Đã hoàn thành" chuyển sang active, tab "Đang diễn ra" hết active; danh sách bên dưới được thay bằng danh sách khác.
-4. Tab "Đang diễn ra" chuyển lại active; danh sách trở về danh sách ban đầu.</t>
+          <t>2. Tab "Đã hoàn thành" chuyển sang active, tab "Đang diễn ra" hết active; danh sách bên dưới được thay bằng danh sách khác.
+3. Tab "Đang diễn ra" chuyển lại active; danh sách trở về danh sách ban đầu.</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>1 đơn "Đang giao" + 1 đơn "Hoàn thành" (test_data_catalog §ACT)</t>
+          <t>Đơn "Đang giao" + đơn "Hoàn thành" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr"/>
@@ -9289,24 +9287,24 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG có ≥1 đơn "Hết hạn".</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment) — gồm đơn "Hết hạn" cần dev/QA chuẩn bị trước vì ⛔ không tạo được qua UI.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed 1 đơn có "Đến ngày" đã trôi qua để đơn chuyển trạng thái "Hết hạn". (setup)
-2. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành".
-3. Check card đơn hết hạn.</t>
+          <t>1. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành". (setup)
+2. Check card đơn "Hết hạn".</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>3. Card hiển thị badge "Hết hạn" và dòng lý do đúng chuỗi "Không có ai nhận mang giúp trong thời gian đăng — tin đã tự động đóng."</t>
+          <t>2. Card hiển thị badge "Hết hạn" và dòng lý do đúng chuỗi "Không có ai nhận mang giúp trong thời gian đăng — tin đã tự động đóng."</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>1 đơn "Hết hạn" (test_data_catalog §ACT — ⛔ không seed được qua UI)</t>
+          <t>Đơn "Hết hạn" của `SEED-ACT-01` (test_data_catalog §ACT — ⛔ không seed được qua UI)</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr"/>
@@ -9365,24 +9363,24 @@
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG có ≥1 đơn "Hết hạn".</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment) — dùng chung đơn "Hết hạn" với TC-ACT-008, không seed lại.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed 1 đơn có "Đến ngày" đã trôi qua để đơn chuyển trạng thái "Hết hạn". (setup)
-2. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành".
-3. Nhấn vào card đơn "Hết hạn".</t>
+          <t>1. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành". (setup)
+2. Nhấn vào card đơn "Hết hạn".</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>3. Không mở màn nào, không hiện popup; màn Hoạt động giữ nguyên với tab "Đã hoàn thành" vẫn active.</t>
+          <t>2. Không mở màn nào, không hiện popup; màn Hoạt động giữ nguyên với tab "Đã hoàn thành" vẫn active.</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>1 đơn "Hết hạn" (test_data_catalog §ACT)</t>
+          <t>Đơn "Hết hạn" của `SEED-ACT-01`, dùng chung với TC-ACT-008 (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr"/>
@@ -9518,7 +9516,8 @@
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản CBNV "trắng" trên STG (không có đơn nào ở trạng thái từ "Chờ ghép" đến "Đã giao").</t>
+          <t>- Tài khoản CBNV "trắng" trên STG = `SEED-ACT-02` (không có đơn nào ở trạng thái từ "Chờ ghép" đến "Đã giao") — dùng chung với TC-ACT-014, chuẩn bị 1 lần.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -9594,24 +9593,24 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG có ≥1 đơn "Hoàn thành".</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment) — dùng chung đơn "Hoàn thành" với TC-ACT-003/005, không seed lại.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed 1 đơn ở trạng thái "Hoàn thành" cho tài khoản. (setup)
-2. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành".
-3. Nhấn vào vùng chuỗi sao trên card đơn "Hoàn thành".</t>
+          <t>1. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành". (setup)
+2. Nhấn vào vùng chuỗi sao trên card đơn "Hoàn thành".</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>3. Không mở màn chấm điểm hay popup chấm sao nào; không có control nào cho phép chọn số sao.</t>
+          <t>2. Không mở màn chấm điểm hay popup chấm sao nào; không có control nào cho phép chọn số sao.</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>1 đơn "Hoàn thành" (test_data_catalog §ACT)</t>
+          <t>Đơn "Hoàn thành" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr"/>
@@ -9670,7 +9669,8 @@
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản CBNV "trắng" trên STG (chưa có đơn "Hoàn thành" và chưa có đơn "Hết hạn").</t>
+          <t>- Tài khoản CBNV "trắng" trên STG = `SEED-ACT-02` (chưa có đơn "Hoàn thành" và chưa có đơn "Hết hạn") — dùng chung với TC-ACT-012, không chuẩn bị lại.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
@@ -24610,7 +24610,7 @@
       <c r="H208" s="6" t="inlineStr">
         <is>
           <t>Tài khoản SSO CBNV FPT còn hiệu lực trên STG.
-- Host app FoxPro (`vn.fpt.ftel.sop.stg`) đã cài trên thiết bị Android.</t>
+- Host app FoxPro (`vn.fpt.ftel.sop.stg`) đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I208" s="6" t="inlineStr">
@@ -25856,26 +25856,26 @@
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG có ≥1 đơn đang hoạt động và ≥1 đơn đã kết thúc.</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment).
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed cho tài khoản 1 đơn ở trạng thái "Đang giao" và 1 đơn ở trạng thái "Hoàn thành". (setup)
-2. Đăng nhập FoxEco và nhấn tab "Hoạt động".
-3. Nhấn tab con "Đã hoàn thành".
-4. Nhấn tab con "Đang diễn ra".</t>
+          <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
+2. Nhấn tab con "Đã hoàn thành".
+3. Nhấn tab con "Đang diễn ra".</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>3. Tab "Đã hoàn thành" chuyển sang active, tab "Đang diễn ra" hết active; danh sách bên dưới được thay bằng danh sách khác.
-4. Tab "Đang diễn ra" chuyển lại active; danh sách trở về danh sách ban đầu.</t>
+          <t>2. Tab "Đã hoàn thành" chuyển sang active, tab "Đang diễn ra" hết active; danh sách bên dưới được thay bằng danh sách khác.
+3. Tab "Đang diễn ra" chuyển lại active; danh sách trở về danh sách ban đầu.</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>1 đơn "Đang giao" + 1 đơn "Hoàn thành" (test_data_catalog §ACT)</t>
+          <t>Đơn "Đang giao" + đơn "Hoàn thành" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L4" s="5" t="inlineStr"/>
@@ -25934,24 +25934,24 @@
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG.</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment).
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed cho tài khoản đủ 4 đơn đang hoạt động ở các trạng thái "Chờ ghép", "Đã ghép", "Đang giao", "Đã giao", cùng 1 đơn "Hoàn thành" và 1 đơn "Hết hạn". (setup)
-2. Đăng nhập FoxEco và nhấn tab "Hoạt động".
-3. Check badge trạng thái của từng card trong tab "Đang diễn ra".</t>
+          <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
+2. Check badge trạng thái của từng card trong tab "Đang diễn ra".</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t>3. Mọi card trong danh sách có badge thuộc nhóm "Chờ ghép", "Đã ghép", "Đang giao", "Đã giao"; KHÔNG có card nào badge "Hoàn thành" hoặc "Hết hạn".</t>
+          <t>2. Mọi card trong danh sách có badge thuộc nhóm "Chờ ghép", "Đã ghép", "Đang giao", "Đã giao"; KHÔNG có card nào badge "Hoàn thành" hoặc "Hết hạn".</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
         <is>
-          <t>4 đơn đang hoạt động + 1 đơn "Hoàn thành" + 1 đơn "Hết hạn" (test_data_catalog §ACT)</t>
+          <t>4 đơn đang hoạt động + 1 đơn "Hoàn thành" + 1 đơn "Hết hạn" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L5" s="7" t="inlineStr"/>
@@ -26010,25 +26010,25 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG.</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment).
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed cho tài khoản 1 đơn "Hoàn thành", 1 đơn "Hết hạn" và 1 đơn "Đang giao". (setup)
-2. Đăng nhập FoxEco và nhấn tab "Hoạt động".
-3. Nhấn tab con "Đã hoàn thành".
-4. Check badge trạng thái của từng card trong danh sách.</t>
+          <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
+2. Nhấn tab con "Đã hoàn thành". (setup)
+3. Check badge trạng thái của từng card trong danh sách.</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>4. Danh sách có card badge "Hoàn thành" và card badge "Hết hạn"; KHÔNG có card nào badge "Chờ ghép", "Đã ghép", "Đang giao" hay "Đã giao".</t>
+          <t>3. Danh sách có card badge "Hoàn thành" và card badge "Hết hạn"; KHÔNG có card nào badge "Chờ ghép", "Đã ghép", "Đang giao" hay "Đã giao".</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>1 đơn "Hoàn thành" + 1 đơn "Hết hạn" + 1 đơn "Đang giao" (test_data_catalog §ACT)</t>
+          <t>1 đơn "Hoàn thành" + 1 đơn "Hết hạn" + 1 đơn "Đang giao" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr"/>
@@ -26087,24 +26087,24 @@
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG có ≥1 đơn đang hoạt động.</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment).
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed cho tài khoản 1 đơn ở trạng thái "Đang giao". (setup)
-2. Đăng nhập FoxEco và nhấn tab "Hoạt động".
-3. Check lần lượt các trường trên card đơn.</t>
+          <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
+2. Check lần lượt các trường trên card đơn "Đang giao".</t>
         </is>
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>3. Card hiển thị đủ 5 trường: icon trạng thái, tên tin, tuyến đường dạng "Từ → Đến", ngày, badge trạng thái.</t>
+          <t>2. Card hiển thị đủ 5 trường: icon trạng thái, tên tin, tuyến đường dạng "Từ → Đến", ngày, badge trạng thái.</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>1 đơn "Đang giao" (test_data_catalog §ACT)</t>
+          <t>Đơn "Đang giao" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L7" s="7" t="inlineStr"/>
@@ -26240,24 +26240,24 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG có ≥1 đơn "Hết hạn".</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment) — gồm đơn "Hết hạn" cần dev/QA chuẩn bị trước vì ⛔ không tạo được qua UI.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed 1 đơn có "Đến ngày" đã trôi qua để đơn chuyển trạng thái "Hết hạn". (setup)
-2. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành".
-3. Check card đơn hết hạn.</t>
+          <t>1. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành". (setup)
+2. Check card đơn "Hết hạn".</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>3. Card hiển thị badge "Hết hạn" và dòng lý do đúng chuỗi "Không có ai nhận mang giúp trong thời gian đăng — tin đã tự động đóng."</t>
+          <t>2. Card hiển thị badge "Hết hạn" và dòng lý do đúng chuỗi "Không có ai nhận mang giúp trong thời gian đăng — tin đã tự động đóng."</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
         <is>
-          <t>1 đơn "Hết hạn" (test_data_catalog §ACT — ⛔ không seed được qua UI)</t>
+          <t>Đơn "Hết hạn" của `SEED-ACT-01` (test_data_catalog §ACT — ⛔ không seed được qua UI)</t>
         </is>
       </c>
       <c r="L9" s="7" t="inlineStr"/>
@@ -26316,24 +26316,24 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG có ≥1 đơn "Hết hạn".</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment) — dùng chung đơn "Hết hạn" với TC-ACT-008, không seed lại.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed 1 đơn có "Đến ngày" đã trôi qua để đơn chuyển trạng thái "Hết hạn". (setup)
-2. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành".
-3. Nhấn vào card đơn "Hết hạn".</t>
+          <t>1. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành". (setup)
+2. Nhấn vào card đơn "Hết hạn".</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>3. Không mở màn nào, không hiện popup; màn Hoạt động giữ nguyên với tab "Đã hoàn thành" vẫn active.</t>
+          <t>2. Không mở màn nào, không hiện popup; màn Hoạt động giữ nguyên với tab "Đã hoàn thành" vẫn active.</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>1 đơn "Hết hạn" (test_data_catalog §ACT)</t>
+          <t>Đơn "Hết hạn" của `SEED-ACT-01`, dùng chung với TC-ACT-008 (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr"/>
@@ -26392,25 +26392,25 @@
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG.</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment) — bất kỳ 2 đơn active nào trong bộ này đã khác tên tin/tuyến sẵn.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed cho tài khoản 2 đơn đang hoạt động khác nhau về tên tin và tuyến đường. (setup)
-2. Đăng nhập FoxEco và nhấn tab "Hoạt động".
-3. Ghi lại tên tin và tuyến đường của card thứ hai.
-4. Nhấn vào card thứ hai.</t>
+          <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
+2. Ghi lại tên tin và tuyến đường của card thứ hai.
+3. Nhấn vào card thứ hai.</t>
         </is>
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>4. Màn vừa mở hiển thị tên tin và tuyến đường trùng khớp thông tin đã ghi ở bước 3.</t>
+          <t>3. Màn vừa mở hiển thị tên tin và tuyến đường trùng khớp thông tin đã ghi ở bước 2.</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
-          <t>2 đơn đang hoạt động khác nhau (test_data_catalog §ACT)</t>
+          <t>2 đơn đang hoạt động khác nhau của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L11" s="7" t="inlineStr"/>
@@ -26546,7 +26546,8 @@
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản CBNV "trắng" trên STG (không có đơn nào ở trạng thái từ "Chờ ghép" đến "Đã giao").</t>
+          <t>- Tài khoản CBNV "trắng" trên STG = `SEED-ACT-02` (không có đơn nào ở trạng thái từ "Chờ ghép" đến "Đã giao") — dùng chung với TC-ACT-014, chuẩn bị 1 lần.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -26622,24 +26623,24 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Tài khoản Sender trên STG có ≥1 đơn "Hoàn thành".</t>
+          <t>- Tài khoản A là CBNV có hồ sơ đầy đủ trên STG, đã seed sẵn `SEED-ACT-01` (xem ghi chú đầu fragment) — dùng chung đơn "Hoàn thành" với TC-ACT-003/005, không seed lại.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>1. Nhờ dev/QA seed 1 đơn ở trạng thái "Hoàn thành" cho tài khoản. (setup)
-2. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành".
-3. Nhấn vào vùng chuỗi sao trên card đơn "Hoàn thành".</t>
+          <t>1. Đăng nhập FoxEco, nhấn tab "Hoạt động" rồi nhấn tab con "Đã hoàn thành". (setup)
+2. Nhấn vào vùng chuỗi sao trên card đơn "Hoàn thành".</t>
         </is>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>3. Không mở màn chấm điểm hay popup chấm sao nào; không có control nào cho phép chọn số sao.</t>
+          <t>2. Không mở màn chấm điểm hay popup chấm sao nào; không có control nào cho phép chọn số sao.</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>1 đơn "Hoàn thành" (test_data_catalog §ACT)</t>
+          <t>Đơn "Hoàn thành" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr"/>
@@ -26698,7 +26699,8 @@
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>Tài khoản CBNV "trắng" trên STG (chưa có đơn "Hoàn thành" và chưa có đơn "Hết hạn").</t>
+          <t>- Tài khoản CBNV "trắng" trên STG = `SEED-ACT-02` (chưa có đơn "Hoàn thành" và chưa có đơn "Hết hạn") — dùng chung với TC-ACT-012, không chuẩn bị lại.
+- Host app FoxPro đã cài trên thiết bị Android/iOS.</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">

</xml_diff>

<commit_message>
test(vibe): execute VR-017 on ACT and VR-018 on CNL [AI]
Record run evidence, scope ledgers and coverage for ACT and CNL,
log BUG-030/031 drafts, sync TC-ACT fragment and TC-MASTER, and
update the STG account registry with data created during the runs.

Refs: N/A
</commit_message>
<xml_diff>
--- a/03_test-cases/TC-MASTER-LATEST.xlsx
+++ b/03_test-cases/TC-MASTER-LATEST.xlsx
@@ -12372,12 +12372,12 @@
           <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
 2. Nhấn tab con "Đã hoàn thành". (setup)
 3. Nhấn tab con "Đang diễn ra" rồi rà toàn bộ danh sách. (setup)
-4. Nhấn lại tab con "Đã hoàn thành" và check cả hai đơn của cặp đối chứng trong cùng một lượt xem.</t>
+4. Nhấn lại tab con "Đã hoàn thành" và check vị trí của cả hai đơn trong cặp đối chứng ở hai tab vừa rà.</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>4. Đơn đã trả lại người gửi CÓ trong danh sách tab "Đã hoàn thành" và hiện lý do hoàn hàng trên card; đơn "Đã huỷ" KHÔNG xuất hiện ở cả hai tab.</t>
+          <t>4. Đơn đã trả lại người gửi CÓ trong danh sách tab "Đã hoàn thành" và hiện lý do hoàn hàng trên card; đơn "Đã huỷ" nằm ở tab "Đang diễn ra" với badge "Đã huỷ" và KHÔNG xuất hiện ở tab "Đã hoàn thành".</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -12388,7 +12388,7 @@
       <c r="L7" s="6" t="inlineStr"/>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: hai kết cục bất thường nhưng hai cách xử lý ngược nhau — giá trị của TC nằm ở **phép đối chứng**, xem lẻ từng đơn thì không bắt được lỗi "gom chung mọi đơn bất thường vào một nhánh hiển thị". · Căn cứ: `AC-24.2.01` cho vế `RETURNED`; vế `CANCELLED` theo BA trả lời `C-ACT-04(b)` 2026-09-17 — đơn "Đã huỷ" **vẫn ẩn khỏi cả 2 tab**, rule v1.0 CÒN HIỆU LỰC, `§8.12.3` cho mọi vai *"Xem lý do"* đơn huỷ là **PRD chưa cập nhật**. Đơn "Đã huỷ" hiện ra ⇒ FAIL và log bug, ⛔ không sửa Expected theo `§8.12.3`. · Phụ thuộc lô `DLV` để có đơn `RETURNED` — lô đó `BLOCKED` thì TC này `BLOCKED`.</t>
+          <t>Đã sửa Expected theo app — QC GiangDC2 chốt 2026-09-21 (sau VR-017): đơn "Đã huỷ" hiện ở tab "Đang diễn ra" với badge "Đã huỷ" là hành vi ĐÚNG, không phải bug; thay kết luận BA `C-ACT-04(b)` 2026-09-17 (ẩn khỏi cả 2 tab). ⚠️ Title chưa sửa vì `§10.5` khoá Title (nợ #27 `03_test-cases/v1.1/CHANGELOG.md`). · Mục đích: hai kết cục bất thường nhưng hai cách xử lý ngược nhau — giá trị của TC nằm ở **phép đối chứng**, xem lẻ từng đơn thì không bắt được lỗi "gom chung mọi đơn bất thường vào một nhánh hiển thị". · Căn cứ: `AC-24.2.01` cho vế `RETURNED`; vế `CANCELLED` theo BA trả lời `C-ACT-04(b)` 2026-09-17 — đơn "Đã huỷ" **vẫn ẩn khỏi cả 2 tab**, rule v1.0 CÒN HIỆU LỰC, `§8.12.3` cho mọi vai *"Xem lý do"* đơn huỷ là **PRD chưa cập nhật**. · Phụ thuộc lô `DLV` để có đơn `RETURNED` — lô đó `BLOCKED` thì TC này `BLOCKED`.</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
@@ -12606,12 +12606,12 @@
 2. Nhấn tab "Hoạt động". (setup)
 3. Vuốt lên và vuốt xuống trên vùng danh sách của tab "Đang diễn ra".
 4. Nhấn tab con "Đã hoàn thành".
-5. Vuốt lên và vuốt xuống trên vùng danh sách, và check phản hồi cuộn của màn ở cả hai tab con.</t>
+5. Vuốt lên và vuốt xuống trên vùng danh sách, và check trạng thái của màn ở cả hai tab con.</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>5. Màn phản hồi thao tác cuộn ở cả hai tab con, không bị khoá cứng tại chỗ.</t>
+          <t>5. Ở cả hai tab con, empty state đứng cố định trong vùng danh sách khi vuốt (nội dung vừa khít màn, không có gì để cuộn); màn không treo, không lỗi và thanh tab dưới vẫn hiển thị đủ.</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -12622,7 +12622,7 @@
       <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.17.2 BR17-03 — rule đòi empty state vừa không che thanh tab dưới vừa giữ màn cuộn được.</t>
+          <t>Đã sửa Expected + step 5 theo app — QC GiangDC2 chốt 2026-09-21 (sau VR-017): màn rỗng không cuộn/không phản hồi vuốt là hành vi ĐÚNG, không phải bug (`BUG-032` đã xoá). ⚠️ Title chưa sửa vì `§10.5` khoá Title (nợ #28 `03_test-cases/v1.1/CHANGELOG.md`). · Căn cứ gốc: `DOC-v1.1-01` §8.17.2 BR17-03 — QC hiểu "vẫn cuộn được" là màn không bị treo/khoá thao tác, không bắt buộc có phản hồi cuộn khi không có nội dung vượt màn.</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
@@ -29946,12 +29946,12 @@
           <t>1. Đăng nhập FoxEco và nhấn tab "Hoạt động". (setup)
 2. Nhấn tab con "Đã hoàn thành". (setup)
 3. Nhấn tab con "Đang diễn ra" rồi rà toàn bộ danh sách. (setup)
-4. Nhấn lại tab con "Đã hoàn thành" và check cả hai đơn của cặp đối chứng trong cùng một lượt xem.</t>
+4. Nhấn lại tab con "Đã hoàn thành" và check vị trí của cả hai đơn trong cặp đối chứng ở hai tab vừa rà.</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>4. Đơn đã trả lại người gửi CÓ trong danh sách tab "Đã hoàn thành" và hiện lý do hoàn hàng trên card; đơn "Đã huỷ" KHÔNG xuất hiện ở cả hai tab.</t>
+          <t>4. Đơn đã trả lại người gửi CÓ trong danh sách tab "Đã hoàn thành" và hiện lý do hoàn hàng trên card; đơn "Đã huỷ" nằm ở tab "Đang diễn ra" với badge "Đã huỷ" và KHÔNG xuất hiện ở tab "Đã hoàn thành".</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -29962,7 +29962,7 @@
       <c r="L6" s="5" t="inlineStr"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: hai kết cục bất thường nhưng hai cách xử lý ngược nhau — giá trị của TC nằm ở **phép đối chứng**, xem lẻ từng đơn thì không bắt được lỗi "gom chung mọi đơn bất thường vào một nhánh hiển thị". · Căn cứ: `AC-24.2.01` cho vế `RETURNED`; vế `CANCELLED` theo BA trả lời `C-ACT-04(b)` 2026-09-17 — đơn "Đã huỷ" **vẫn ẩn khỏi cả 2 tab**, rule v1.0 CÒN HIỆU LỰC, `§8.12.3` cho mọi vai *"Xem lý do"* đơn huỷ là **PRD chưa cập nhật**. Đơn "Đã huỷ" hiện ra ⇒ FAIL và log bug, ⛔ không sửa Expected theo `§8.12.3`. · Phụ thuộc lô `DLV` để có đơn `RETURNED` — lô đó `BLOCKED` thì TC này `BLOCKED`.</t>
+          <t>Đã sửa Expected theo app — QC GiangDC2 chốt 2026-09-21 (sau VR-017): đơn "Đã huỷ" hiện ở tab "Đang diễn ra" với badge "Đã huỷ" là hành vi ĐÚNG, không phải bug; thay kết luận BA `C-ACT-04(b)` 2026-09-17 (ẩn khỏi cả 2 tab). ⚠️ Title chưa sửa vì `§10.5` khoá Title (nợ #27 `03_test-cases/v1.1/CHANGELOG.md`). · Mục đích: hai kết cục bất thường nhưng hai cách xử lý ngược nhau — giá trị của TC nằm ở **phép đối chứng**, xem lẻ từng đơn thì không bắt được lỗi "gom chung mọi đơn bất thường vào một nhánh hiển thị". · Căn cứ: `AC-24.2.01` cho vế `RETURNED`; vế `CANCELLED` theo BA trả lời `C-ACT-04(b)` 2026-09-17 — đơn "Đã huỷ" **vẫn ẩn khỏi cả 2 tab**, rule v1.0 CÒN HIỆU LỰC, `§8.12.3` cho mọi vai *"Xem lý do"* đơn huỷ là **PRD chưa cập nhật**. · Phụ thuộc lô `DLV` để có đơn `RETURNED` — lô đó `BLOCKED` thì TC này `BLOCKED`.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
@@ -30439,12 +30439,12 @@
 2. Nhấn tab "Hoạt động". (setup)
 3. Vuốt lên và vuốt xuống trên vùng danh sách của tab "Đang diễn ra".
 4. Nhấn tab con "Đã hoàn thành".
-5. Vuốt lên và vuốt xuống trên vùng danh sách, và check phản hồi cuộn của màn ở cả hai tab con.</t>
+5. Vuốt lên và vuốt xuống trên vùng danh sách, và check trạng thái của màn ở cả hai tab con.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>5. Màn phản hồi thao tác cuộn ở cả hai tab con, không bị khoá cứng tại chỗ.</t>
+          <t>5. Ở cả hai tab con, empty state đứng cố định trong vùng danh sách khi vuốt (nội dung vừa khít màn, không có gì để cuộn); màn không treo, không lỗi và thanh tab dưới vẫn hiển thị đủ.</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -30455,7 +30455,7 @@
       <c r="L16" s="5" t="inlineStr"/>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.17.2 BR17-03 — rule đòi empty state vừa không che thanh tab dưới vừa giữ màn cuộn được.</t>
+          <t>Đã sửa Expected + step 5 theo app — QC GiangDC2 chốt 2026-09-21 (sau VR-017): màn rỗng không cuộn/không phản hồi vuốt là hành vi ĐÚNG, không phải bug (`BUG-032` đã xoá). ⚠️ Title chưa sửa vì `§10.5` khoá Title (nợ #28 `03_test-cases/v1.1/CHANGELOG.md`). · Căn cứ gốc: `DOC-v1.1-01` §8.17.2 BR17-03 — QC hiểu "vẫn cuộn được" là màn không bị treo/khoá thao tác, không bắt buộc có phản hồi cuộn khi không có nội dung vượt màn.</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">

</xml_diff>

<commit_message>
test(tc): align DLV return-flow cases with QC decisions [AI]
A Playwright check of the three-role demo showed the RESCHEDULED and
RETURNING screens exist but use different wording, and that PRD
§8.12.3 only quotes real button labels; unquoted cells describe what
a role can do. TC-DLV-031..036 now assert that meaning instead of
exact text.

QC decisions applied (2026-09-23): only the sender closes a returning
order, with the PRD label "Xác nhận đã nhận lại hàng"; the closed
order shows "Hoàn thành" (TC-DLV-063). Tab, "Xem lý do"/"Đăng lại",
gift and log wording keep the current PRD-based expectations. The
export sheet is re-patched in column I only (I8-I13, I45); results
and every other sheet are untouched. Case count stays 223 (DLV 51).

Refs: N/A

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_test-cases/TC-MASTER-LATEST.xlsx
+++ b/03_test-cases/TC-MASTER-LATEST.xlsx
@@ -15539,7 +15539,7 @@
       <c r="L40" s="5" t="n"/>
       <c r="M40" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: oracle bảo vệ ranh giới `RETURNED` ⟷ `COMPLETED` — lỗi hay gặp nhất là coi hoàn hàng như một dạng hoàn thành. Chạy sớm nhất trong nhóm hậu-hoàn-hàng. · Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06 + §8.14.1 (bước tặng quà chỉ mở ở đơn Hoàn thành). Cặp với TC-DLV-065. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Chạy CHUNG với TC-DLV-063 (1 lần xác nhận, 2 evidence). Demo có nút "Cảm ơn người vận chuyển" ở đơn trả hàng — gặp trên STG ⇒ FAIL.</t>
+          <t>Mục đích: oracle bảo vệ ranh giới `RETURNED` ⟷ `COMPLETED` — lỗi hay gặp nhất là coi hoàn hàng như một dạng hoàn thành. Chạy sớm nhất trong nhóm hậu-hoàn-hàng. · Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06 + §8.14.1 (bước tặng quà chỉ mở ở đơn Hoàn thành). Cặp với TC-DLV-065. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Chạy CHUNG với TC-DLV-063 (1 lần xác nhận, 2 evidence). Demo có nút "Cảm ơn người vận chuyển" ở đơn trả hàng — gặp trên STG ⇒ FAIL. ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N40" s="5" t="inlineStr">
@@ -15616,7 +15616,7 @@
       <c r="L41" s="6" t="n"/>
       <c r="M41" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: điểm fail độc lập với TC-DLV-064 — bước tặng quà và chỉ số đóng góp là hai bề mặt khác nhau, khoá một bề mặt không đảm bảo khoá bề mặt kia. · Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06. Đơn vẫn phải xuất hiện trong tab "Đã hoàn thành" — verify ở TC-DLV-063. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận").</t>
+          <t>Mục đích: điểm fail độc lập với TC-DLV-064 — bước tặng quà và chỉ số đóng góp là hai bề mặt khác nhau, khoá một bề mặt không đảm bảo khoá bề mặt kia. · Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06. Đơn vẫn phải xuất hiện trong tab "Đã hoàn thành" — verify ở TC-DLV-063. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N41" s="6" t="inlineStr">
@@ -16011,7 +16011,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Xem lịch hẹn giao lại".</t>
+          <t>3. Màn Theo dõi đơn của người gửi hiển thị lịch hẹn giao lại (ngày · khoảng giờ · nơi giao lại) và người gửi KHÔNG có nút hành động nào để đổi trạng thái đơn.</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
@@ -16022,7 +16022,7 @@
       <c r="L46" s="5" t="n"/>
       <c r="M46" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: 1 trong 3 ô vai của nhóm trạng thái `RESCHEDULED` — mỗi vai fail độc lập. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED. ⚠ Thanh timeline vẫn hiện đúng 5 mốc và mốc "Đang giao" đang active — đây là thiết kế đã chốt (`C-DLV-05(d)` Resolved 2026-09-17), ⛔ không FAIL vì thiếu mốc mới. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. (demo: "Người vận chuyển đang giữ hàng · sẽ giao lại theo lịch hẹn").</t>
+          <t>Mục đích: 1 trong 3 ô vai của nhóm trạng thái `RESCHEDULED` — mỗi vai fail độc lập. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED. ⚠ Thanh timeline vẫn hiện đúng 5 mốc và mốc "Đang giao" đang active — đây là thiết kế đã chốt (`C-DLV-05(d)` Resolved 2026-09-17), ⛔ không FAIL vì thiếu mốc mới. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Expected so theo NGHĨA: PRD §8.12.3 chỉ đặt trong ngoặc kép những chữ là nhãn nút thật; ô này KHÔNG có ngoặc kép ⇒ là mô tả việc vai đó làm được, ⛔ không đòi đúng từng chữ. Ghi nguyên văn nhãn STG vào Notes. Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): khối "Sẽ giao lại cho người nhận" + nút xám "Người vận chuyển đang giữ hàng · sẽ giao lại theo lịch hẹn" ⇒ thoả.</t>
         </is>
       </c>
       <c r="N46" s="5" t="inlineStr">
@@ -16088,7 +16088,7 @@
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Giao lại theo lịch" ở trạng thái enable.</t>
+          <t>3. Nút hành động chính của người vận chuyển ở trạng thái enable và là hành động giao lại cho người nhận (mở lại màn giao hàng khi nhấn — việc nhấn thuộc TC-DLV-062).</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
@@ -16099,7 +16099,7 @@
       <c r="L47" s="6" t="n"/>
       <c r="M47" s="6" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED — đây là vai DUY NHẤT có nút hành động thật ở trạng thái này, 2 vai kia chỉ xem. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Bỏ vế "nhấn được để mở lại màn giao hàng" khỏi Expected vì nhấn sẽ tiêu trạng thái của TC-DLV-031/033/072 — vế này đã do TC-DLV-062 phủ. Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. (demo: "Giao lại cho người nhận").</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED — đây là vai DUY NHẤT có nút hành động thật ở trạng thái này, 2 vai kia chỉ xem. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Expected so theo NGHĨA: PRD §8.12.3 chỉ đặt trong ngoặc kép những chữ là nhãn nút thật; ô này KHÔNG có ngoặc kép ⇒ là mô tả việc vai đó làm được, ⛔ không đòi đúng từng chữ. Ghi nguyên văn nhãn STG vào Notes. Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): nút cam "Giao lại cho người nhận" ⇒ thoả. Bỏ vế "nhấn được" khỏi TC này vì nhấn sẽ tiêu trạng thái của TC-DLV-031/033/072.</t>
         </is>
       </c>
       <c r="N47" s="6" t="inlineStr">
@@ -16165,7 +16165,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Xem lịch hẹn" và KHÔNG có nút giao lại nào.</t>
+          <t>3. Màn Theo dõi đơn của người nhận hiển thị lịch hẹn giao lại (ngày · khoảng giờ · nơi) và người nhận KHÔNG có nút giao lại hay nút hành động nào.</t>
         </is>
       </c>
       <c r="K48" s="5" t="inlineStr">
@@ -16176,7 +16176,7 @@
       <c r="L48" s="5" t="n"/>
       <c r="M48" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: đối chứng với TC-DLV-032 — quyền giao lại chỉ thuộc người vận chuyển. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. (demo: "Người vận chuyển sẽ giao lại theo lịch hẹn").</t>
+          <t>Mục đích: đối chứng với TC-DLV-032 — quyền giao lại chỉ thuộc người vận chuyển. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Expected so theo NGHĨA: PRD §8.12.3 chỉ đặt trong ngoặc kép những chữ là nhãn nút thật; ô này KHÔNG có ngoặc kép ⇒ là mô tả việc vai đó làm được, ⛔ không đòi đúng từng chữ. Ghi nguyên văn nhãn STG vào Notes. Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): khối lịch hẹn + nút xám "Người vận chuyển sẽ giao lại theo lịch hẹn" ⇒ thoả.</t>
         </is>
       </c>
       <c r="N48" s="5" t="inlineStr">
@@ -16242,7 +16242,7 @@
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Xác nhận đã nhận lại hàng" ở trạng thái enable và màn có mục xem lịch hẹn trả hàng.</t>
+          <t>3. Nút hành động chính hiển thị đúng chữ "Xác nhận đã nhận lại hàng" ở trạng thái enable và màn hiển thị lịch hẹn trả hàng (ngày · khoảng giờ · nơi).</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
@@ -16253,7 +16253,7 @@
       <c r="L49" s="6" t="n"/>
       <c r="M49" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: người gửi là vai DUY NHẤT đóng được đơn ở nhánh hoàn hàng — cặp với TC-DLV-063. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. (demo: "Đã lấy lại hàng từ người giao").</t>
+          <t>Mục đích: người gửi là vai DUY NHẤT đóng được đơn ở nhánh hoàn hàng — cặp với TC-DLV-063. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23 (theo PRD): CHỈ người gửi đóng đơn trả hàng, nhãn nút đúng chữ "Xác nhận đã nhận lại hàng"; đơn sau khi người gửi nhận lại hiển thị trạng thái "Hoàn thành". Demo ghi "Đã lấy lại hàng từ người giao" ⇒ STG giống demo = FAIL + log bug dẫn §8.12.3. Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): khối "Đơn chuyển sang trả hàng" có lịch hẹn.</t>
         </is>
       </c>
       <c r="N49" s="6" t="inlineStr">
@@ -16319,7 +16319,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Xem lịch hẹn trả hàng" và KHÔNG có nút xác nhận đóng đơn.</t>
+          <t>3. Màn Theo dõi đơn của người vận chuyển hiển thị lịch hẹn trả hàng (ngày · khoảng giờ · nơi) và KHÔNG có nút xác nhận đã trả hàng / đóng đơn nào.</t>
         </is>
       </c>
       <c r="K50" s="5" t="inlineStr">
@@ -16330,7 +16330,7 @@
       <c r="L50" s="5" t="n"/>
       <c r="M50" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. ⚠ Demo cho B nút "Đã trả hàng cho người gửi" (ngược Expected) — gặp trên STG ⇒ FAIL + log bug dẫn §8.12.3.</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23 (theo PRD): CHỈ người gửi đóng đơn trả hàng, nhãn nút đúng chữ "Xác nhận đã nhận lại hàng"; đơn sau khi người gửi nhận lại hiển thị trạng thái "Hoàn thành". Người vận chuyển KHÔNG có nút đóng/xác nhận trả hàng. Expected so theo NGHĨA: PRD §8.12.3 chỉ đặt trong ngoặc kép những chữ là nhãn nút thật; ô này KHÔNG có ngoặc kép ⇒ là mô tả việc vai đó làm được, ⛔ không đòi đúng từng chữ. Ghi nguyên văn nhãn STG vào Notes. ⚠ Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): người vận chuyển CÓ nút cam "Đã trả hàng cho người gửi" ⇒ trái quyết định trên; STG giống demo ⇒ FAIL + log bug dẫn §8.12.3 + quyết định QC 2026-09-23.</t>
         </is>
       </c>
       <c r="N50" s="5" t="inlineStr">
@@ -16396,7 +16396,7 @@
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Xem lý do hoàn hàng".</t>
+          <t>3. Màn Theo dõi đơn của người nhận cho biết đơn không giao được và đang được trả lại người gửi, hiển thị lý do/ghi chú của người vận chuyển, và người nhận KHÔNG có nút hành động nào.</t>
         </is>
       </c>
       <c r="K51" s="6" t="inlineStr">
@@ -16407,7 +16407,7 @@
       <c r="L51" s="6" t="n"/>
       <c r="M51" s="6" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. (demo: "Không giao được · hàng đang được trả lại người gửi").</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Expected so theo NGHĨA: PRD §8.12.3 chỉ đặt trong ngoặc kép những chữ là nhãn nút thật; ô này KHÔNG có ngoặc kép ⇒ là mô tả việc vai đó làm được, ⛔ không đòi đúng từng chữ. Ghi nguyên văn nhãn STG vào Notes. Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): khối "Đơn chuyển sang trả hàng" + ghi chú "Người nhận từ chối nhận hàng" + nút xám "Không giao được · hàng đang được trả lại người gửi" ⇒ thoả.</t>
         </is>
       </c>
       <c r="N51" s="6" t="inlineStr">
@@ -17611,7 +17611,7 @@
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>4. Đơn nằm ở tab "Đã hoàn thành", nhãn trạng thái KHÔNG phải "Hoàn thành" (đơn trả người gửi khác đơn hoàn thành — BR09-06) và nút "Xác nhận đã nhận lại hàng" không còn.</t>
+          <t>4. Đơn hiển thị nhãn trạng thái "Hoàn thành", nút "Xác nhận đã nhận lại hàng" không còn, và đơn nằm ở tab "Đã hoàn thành".</t>
         </is>
       </c>
       <c r="K66" s="5" t="inlineStr">
@@ -17622,7 +17622,7 @@
       <c r="L66" s="5" t="n"/>
       <c r="M66" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06. Đây là bước tạo trạng thái `RETURNED` dùng chung cho TC-DLV-037/038/039, TC-DLV-064/065, TC-DLV-073 và cho `GIFT`/`ACT` — chạy xong mới chạy nhóm đó. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Ghi nguyên văn nhãn trạng thái STG hiển thị vào Notes (PRD không đặc tả chữ). ⚠ Demo 2026-09-23 lệch PRD: cần CẢ B bấm "Đã trả hàng cho người gửi" và A bấm "Đã lấy lại hàng từ người giao", rồi đơn thành "Hoàn thành" — STG làm như demo ⇒ FAIL + log bug dẫn BR09-06.</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06. Đây là bước tạo trạng thái `RETURNED` dùng chung cho TC-DLV-037/038/039, TC-DLV-064/065, TC-DLV-073 và cho `GIFT`/`ACT` — chạy xong mới chạy nhóm đó. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23 (theo PRD): CHỈ người gửi đóng đơn trả hàng, nhãn nút đúng chữ "Xác nhận đã nhận lại hàng"; đơn sau khi người gửi nhận lại hiển thị trạng thái "Hoàn thành". ⇒ Expected đổi từ "KHÔNG phải Hoàn thành" sang nhãn "Hoàn thành" (khác cách đọc BR09-06 trước đây; phần "không mở tặng quà / không cộng Đơn đã giúp" vẫn assert ở TC-DLV-064/065). Tab chứa đơn "Đã hoàn thành": QC chốt giữ nguyên 2026-09-23. ⚠ Demo bắt CẢ 2 bên xác nhận mới đóng — trái quyết định trên; STG giống demo ⇒ FAIL + log bug.</t>
         </is>
       </c>
       <c r="N66" s="5" t="inlineStr">
@@ -18171,7 +18171,7 @@
       <c r="L73" s="6" t="n"/>
       <c r="M73" s="6" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.12.4 mẫu câu 6 — mẫu câu duy nhất do người gửi kích hoạt, 5 mẫu còn lại do người vận chuyển. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ⚠ Demo ghi "Người gửi xác nhận đã nhận lại hàng" / "Đơn đóng · hàng đã về người gửi" — khác PRD §8.12.4; STG lệch ⇒ log bug.</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.12.4 mẫu câu 6 — mẫu câu duy nhất do người gửi kích hoạt, 5 mẫu còn lại do người vận chuyển. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ⚠ Demo ghi "Người gửi xác nhận đã nhận lại hàng" / "Đơn đóng · hàng đã về người gửi" — khác PRD §8.12.4; STG lệch ⇒ log bug. ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N73" s="6" t="inlineStr">
@@ -18249,7 +18249,7 @@
       <c r="L74" s="5" t="n"/>
       <c r="M74" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: nhóm ba trạng thái đóng phải cho CÙNG một nhãn — lệch giữa ba đơn mới là defect. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng (PRD chỉ mô tả cấp danh mục, không có microcopy riêng cho từng trạng thái). · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Đơn hết hạn lấy từ tin cũ có sẵn trên STG, ⛔ không chờ dev. Thiếu đơn hết hạn ⇒ verdict chỉ dựa trên 2 đơn, ghi rõ trong Notes.</t>
+          <t>Mục đích: nhóm ba trạng thái đóng phải cho CÙNG một nhãn — lệch giữa ba đơn mới là defect. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng (PRD chỉ mô tả cấp danh mục, không có microcopy riêng cho từng trạng thái). · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Đơn hết hạn lấy từ tin cũ có sẵn trên STG, ⛔ không chờ dev. Thiếu đơn hết hạn ⇒ verdict chỉ dựa trên 2 đơn, ghi rõ trong Notes. ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N74" s="5" t="inlineStr">
@@ -18326,7 +18326,7 @@
       <c r="L75" s="6" t="n"/>
       <c r="M75" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: đối chứng với TC-DLV-037 — quyền đăng lại chỉ thuộc người gửi. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận").</t>
+          <t>Mục đích: đối chứng với TC-DLV-037 — quyền đăng lại chỉ thuộc người gửi. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N75" s="6" t="inlineStr">
@@ -18403,7 +18403,7 @@
       <c r="L76" s="5" t="n"/>
       <c r="M76" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận").</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N76" s="5" t="inlineStr">
@@ -34230,7 +34230,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Xem lịch hẹn giao lại".</t>
+          <t>3. Màn Theo dõi đơn của người gửi hiển thị lịch hẹn giao lại (ngày · khoảng giờ · nơi giao lại) và người gửi KHÔNG có nút hành động nào để đổi trạng thái đơn.</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -34241,7 +34241,7 @@
       <c r="L3" s="5" t="n"/>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: 1 trong 3 ô vai của nhóm trạng thái `RESCHEDULED` — mỗi vai fail độc lập. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED. ⚠ Thanh timeline vẫn hiện đúng 5 mốc và mốc "Đang giao" đang active — đây là thiết kế đã chốt (`C-DLV-05(d)` Resolved 2026-09-17), ⛔ không FAIL vì thiếu mốc mới. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. (demo: "Người vận chuyển đang giữ hàng · sẽ giao lại theo lịch hẹn").</t>
+          <t>Mục đích: 1 trong 3 ô vai của nhóm trạng thái `RESCHEDULED` — mỗi vai fail độc lập. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED. ⚠ Thanh timeline vẫn hiện đúng 5 mốc và mốc "Đang giao" đang active — đây là thiết kế đã chốt (`C-DLV-05(d)` Resolved 2026-09-17), ⛔ không FAIL vì thiếu mốc mới. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Expected so theo NGHĨA: PRD §8.12.3 chỉ đặt trong ngoặc kép những chữ là nhãn nút thật; ô này KHÔNG có ngoặc kép ⇒ là mô tả việc vai đó làm được, ⛔ không đòi đúng từng chữ. Ghi nguyên văn nhãn STG vào Notes. Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): khối "Sẽ giao lại cho người nhận" + nút xám "Người vận chuyển đang giữ hàng · sẽ giao lại theo lịch hẹn" ⇒ thoả.</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr">
@@ -34307,7 +34307,7 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Giao lại theo lịch" ở trạng thái enable.</t>
+          <t>3. Nút hành động chính của người vận chuyển ở trạng thái enable và là hành động giao lại cho người nhận (mở lại màn giao hàng khi nhấn — việc nhấn thuộc TC-DLV-062).</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
@@ -34318,7 +34318,7 @@
       <c r="L4" s="6" t="n"/>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED — đây là vai DUY NHẤT có nút hành động thật ở trạng thái này, 2 vai kia chỉ xem. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Bỏ vế "nhấn được để mở lại màn giao hàng" khỏi Expected vì nhấn sẽ tiêu trạng thái của TC-DLV-031/033/072 — vế này đã do TC-DLV-062 phủ. Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. (demo: "Giao lại cho người nhận").</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED — đây là vai DUY NHẤT có nút hành động thật ở trạng thái này, 2 vai kia chỉ xem. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Expected so theo NGHĨA: PRD §8.12.3 chỉ đặt trong ngoặc kép những chữ là nhãn nút thật; ô này KHÔNG có ngoặc kép ⇒ là mô tả việc vai đó làm được, ⛔ không đòi đúng từng chữ. Ghi nguyên văn nhãn STG vào Notes. Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): nút cam "Giao lại cho người nhận" ⇒ thoả. Bỏ vế "nhấn được" khỏi TC này vì nhấn sẽ tiêu trạng thái của TC-DLV-031/033/072.</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
@@ -34384,7 +34384,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Xem lịch hẹn" và KHÔNG có nút giao lại nào.</t>
+          <t>3. Màn Theo dõi đơn của người nhận hiển thị lịch hẹn giao lại (ngày · khoảng giờ · nơi) và người nhận KHÔNG có nút giao lại hay nút hành động nào.</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -34395,7 +34395,7 @@
       <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: đối chứng với TC-DLV-032 — quyền giao lại chỉ thuộc người vận chuyển. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. (demo: "Người vận chuyển sẽ giao lại theo lịch hẹn").</t>
+          <t>Mục đích: đối chứng với TC-DLV-032 — quyền giao lại chỉ thuộc người vận chuyển. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RESCHEDULED. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Expected so theo NGHĨA: PRD §8.12.3 chỉ đặt trong ngoặc kép những chữ là nhãn nút thật; ô này KHÔNG có ngoặc kép ⇒ là mô tả việc vai đó làm được, ⛔ không đòi đúng từng chữ. Ghi nguyên văn nhãn STG vào Notes. Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): khối lịch hẹn + nút xám "Người vận chuyển sẽ giao lại theo lịch hẹn" ⇒ thoả.</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr">
@@ -34461,7 +34461,7 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Xác nhận đã nhận lại hàng" ở trạng thái enable và màn có mục xem lịch hẹn trả hàng.</t>
+          <t>3. Nút hành động chính hiển thị đúng chữ "Xác nhận đã nhận lại hàng" ở trạng thái enable và màn hiển thị lịch hẹn trả hàng (ngày · khoảng giờ · nơi).</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -34472,7 +34472,7 @@
       <c r="L6" s="6" t="n"/>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: người gửi là vai DUY NHẤT đóng được đơn ở nhánh hoàn hàng — cặp với TC-DLV-063. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. (demo: "Đã lấy lại hàng từ người giao").</t>
+          <t>Mục đích: người gửi là vai DUY NHẤT đóng được đơn ở nhánh hoàn hàng — cặp với TC-DLV-063. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23 (theo PRD): CHỈ người gửi đóng đơn trả hàng, nhãn nút đúng chữ "Xác nhận đã nhận lại hàng"; đơn sau khi người gửi nhận lại hiển thị trạng thái "Hoàn thành". Demo ghi "Đã lấy lại hàng từ người giao" ⇒ STG giống demo = FAIL + log bug dẫn §8.12.3. Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): khối "Đơn chuyển sang trả hàng" có lịch hẹn.</t>
         </is>
       </c>
       <c r="N6" s="6" t="inlineStr">
@@ -34538,7 +34538,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Xem lịch hẹn trả hàng" và KHÔNG có nút xác nhận đóng đơn.</t>
+          <t>3. Màn Theo dõi đơn của người vận chuyển hiển thị lịch hẹn trả hàng (ngày · khoảng giờ · nơi) và KHÔNG có nút xác nhận đã trả hàng / đóng đơn nào.</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -34549,7 +34549,7 @@
       <c r="L7" s="5" t="n"/>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. ⚠ Demo cho B nút "Đã trả hàng cho người gửi" (ngược Expected) — gặp trên STG ⇒ FAIL + log bug dẫn §8.12.3.</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23 (theo PRD): CHỈ người gửi đóng đơn trả hàng, nhãn nút đúng chữ "Xác nhận đã nhận lại hàng"; đơn sau khi người gửi nhận lại hiển thị trạng thái "Hoàn thành". Người vận chuyển KHÔNG có nút đóng/xác nhận trả hàng. Expected so theo NGHĨA: PRD §8.12.3 chỉ đặt trong ngoặc kép những chữ là nhãn nút thật; ô này KHÔNG có ngoặc kép ⇒ là mô tả việc vai đó làm được, ⛔ không đòi đúng từng chữ. Ghi nguyên văn nhãn STG vào Notes. ⚠ Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): người vận chuyển CÓ nút cam "Đã trả hàng cho người gửi" ⇒ trái quyết định trên; STG giống demo ⇒ FAIL + log bug dẫn §8.12.3 + quyết định QC 2026-09-23.</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr">
@@ -34615,7 +34615,7 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>3. Nhãn hành động chính hiển thị "Xem lý do hoàn hàng".</t>
+          <t>3. Màn Theo dõi đơn của người nhận cho biết đơn không giao được và đang được trả lại người gửi, hiển thị lý do/ghi chú của người vận chuyển, và người nhận KHÔNG có nút hành động nào.</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -34626,7 +34626,7 @@
       <c r="L8" s="6" t="n"/>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Demo 2026-09-23 hiện nhãn KHÁC PRD §8.12.3 ở nhóm trạng thái mới — oracle vẫn theo PRD; STG hiện chữ nào thì ghi nguyên văn vào Notes, lệch PRD ⇒ log bug dẫn §8.12.3, ⛔ không sửa Expected theo demo. (demo: "Không giao được · hàng đang được trả lại người gửi").</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng RETURNING. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Expected so theo NGHĨA: PRD §8.12.3 chỉ đặt trong ngoặc kép những chữ là nhãn nút thật; ô này KHÔNG có ngoặc kép ⇒ là mô tả việc vai đó làm được, ⛔ không đòi đúng từng chữ. Ghi nguyên văn nhãn STG vào Notes. Đã đối chiếu demo bằng Playwright 2026-09-23 (3 vai cùng lúc): khối "Đơn chuyển sang trả hàng" + ghi chú "Người nhận từ chối nhận hàng" + nút xám "Không giao được · hàng đang được trả lại người gửi" ⇒ thoả.</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
@@ -34704,7 +34704,7 @@
       <c r="L9" s="5" t="n"/>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: nhóm ba trạng thái đóng phải cho CÙNG một nhãn — lệch giữa ba đơn mới là defect. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng (PRD chỉ mô tả cấp danh mục, không có microcopy riêng cho từng trạng thái). · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Đơn hết hạn lấy từ tin cũ có sẵn trên STG, ⛔ không chờ dev. Thiếu đơn hết hạn ⇒ verdict chỉ dựa trên 2 đơn, ghi rõ trong Notes.</t>
+          <t>Mục đích: nhóm ba trạng thái đóng phải cho CÙNG một nhãn — lệch giữa ba đơn mới là defect. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng (PRD chỉ mô tả cấp danh mục, không có microcopy riêng cho từng trạng thái). · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Đơn hết hạn lấy từ tin cũ có sẵn trên STG, ⛔ không chờ dev. Thiếu đơn hết hạn ⇒ verdict chỉ dựa trên 2 đơn, ghi rõ trong Notes. ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr">
@@ -34781,7 +34781,7 @@
       <c r="L10" s="6" t="n"/>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: đối chứng với TC-DLV-037 — quyền đăng lại chỉ thuộc người gửi. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận").</t>
+          <t>Mục đích: đối chứng với TC-DLV-037 — quyền đăng lại chỉ thuộc người gửi. · Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
@@ -34858,7 +34858,7 @@
       <c r="L11" s="5" t="n"/>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận").</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.12.3 dòng nhóm đóng. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr">
@@ -36829,7 +36829,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>4. Đơn nằm ở tab "Đã hoàn thành", nhãn trạng thái KHÔNG phải "Hoàn thành" (đơn trả người gửi khác đơn hoàn thành — BR09-06) và nút "Xác nhận đã nhận lại hàng" không còn.</t>
+          <t>4. Đơn hiển thị nhãn trạng thái "Hoàn thành", nút "Xác nhận đã nhận lại hàng" không còn, và đơn nằm ở tab "Đã hoàn thành".</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
@@ -36840,7 +36840,7 @@
       <c r="L40" s="5" t="n"/>
       <c r="M40" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06. Đây là bước tạo trạng thái `RETURNED` dùng chung cho TC-DLV-037/038/039, TC-DLV-064/065, TC-DLV-073 và cho `GIFT`/`ACT` — chạy xong mới chạy nhóm đó. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Ghi nguyên văn nhãn trạng thái STG hiển thị vào Notes (PRD không đặc tả chữ). ⚠ Demo 2026-09-23 lệch PRD: cần CẢ B bấm "Đã trả hàng cho người gửi" và A bấm "Đã lấy lại hàng từ người giao", rồi đơn thành "Hoàn thành" — STG làm như demo ⇒ FAIL + log bug dẫn BR09-06.</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06. Đây là bước tạo trạng thái `RETURNED` dùng chung cho TC-DLV-037/038/039, TC-DLV-064/065, TC-DLV-073 và cho `GIFT`/`ACT` — chạy xong mới chạy nhóm đó. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23 (theo PRD): CHỈ người gửi đóng đơn trả hàng, nhãn nút đúng chữ "Xác nhận đã nhận lại hàng"; đơn sau khi người gửi nhận lại hiển thị trạng thái "Hoàn thành". ⇒ Expected đổi từ "KHÔNG phải Hoàn thành" sang nhãn "Hoàn thành" (khác cách đọc BR09-06 trước đây; phần "không mở tặng quà / không cộng Đơn đã giúp" vẫn assert ở TC-DLV-064/065). Tab chứa đơn "Đã hoàn thành": QC chốt giữ nguyên 2026-09-23. ⚠ Demo bắt CẢ 2 bên xác nhận mới đóng — trái quyết định trên; STG giống demo ⇒ FAIL + log bug.</t>
         </is>
       </c>
       <c r="N40" s="5" t="inlineStr">
@@ -36918,7 +36918,7 @@
       <c r="L41" s="6" t="n"/>
       <c r="M41" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: oracle bảo vệ ranh giới `RETURNED` ⟷ `COMPLETED` — lỗi hay gặp nhất là coi hoàn hàng như một dạng hoàn thành. Chạy sớm nhất trong nhóm hậu-hoàn-hàng. · Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06 + §8.14.1 (bước tặng quà chỉ mở ở đơn Hoàn thành). Cặp với TC-DLV-065. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Chạy CHUNG với TC-DLV-063 (1 lần xác nhận, 2 evidence). Demo có nút "Cảm ơn người vận chuyển" ở đơn trả hàng — gặp trên STG ⇒ FAIL.</t>
+          <t>Mục đích: oracle bảo vệ ranh giới `RETURNED` ⟷ `COMPLETED` — lỗi hay gặp nhất là coi hoàn hàng như một dạng hoàn thành. Chạy sớm nhất trong nhóm hậu-hoàn-hàng. · Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06 + §8.14.1 (bước tặng quà chỉ mở ở đơn Hoàn thành). Cặp với TC-DLV-065. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). Chạy CHUNG với TC-DLV-063 (1 lần xác nhận, 2 evidence). Demo có nút "Cảm ơn người vận chuyển" ở đơn trả hàng — gặp trên STG ⇒ FAIL. ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N41" s="6" t="inlineStr">
@@ -36995,7 +36995,7 @@
       <c r="L42" s="5" t="n"/>
       <c r="M42" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: điểm fail độc lập với TC-DLV-064 — bước tặng quà và chỉ số đóng góp là hai bề mặt khác nhau, khoá một bề mặt không đảm bảo khoá bề mặt kia. · Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06. Đơn vẫn phải xuất hiện trong tab "Đã hoàn thành" — verify ở TC-DLV-063. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận").</t>
+          <t>Mục đích: điểm fail độc lập với TC-DLV-064 — bước tặng quà và chỉ số đóng góp là hai bề mặt khác nhau, khoá một bề mặt không đảm bảo khoá bề mặt kia. · Căn cứ: `DOC-v1.1-01` §8.9.1 BR09-06. Đơn vẫn phải xuất hiện trong tab "Đã hoàn thành" — verify ở TC-DLV-063. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N42" s="5" t="inlineStr">
@@ -37633,7 +37633,7 @@
       <c r="L51" s="5" t="n"/>
       <c r="M51" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §8.12.4 mẫu câu 6 — mẫu câu duy nhất do người gửi kích hoạt, 5 mẫu còn lại do người vận chuyển. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ⚠ Demo ghi "Người gửi xác nhận đã nhận lại hàng" / "Đơn đóng · hàng đã về người gửi" — khác PRD §8.12.4; STG lệch ⇒ log bug.</t>
+          <t>Căn cứ: `DOC-v1.1-01` §8.12.4 mẫu câu 6 — mẫu câu duy nhất do người gửi kích hoạt, 5 mẫu còn lại do người vận chuyển. · 🔁 Sửa 2026-09-23 (QC): Steps chuẩn hoá: dùng đơn seed thay vì tạo đơn mới mỗi TC; ghi rõ 2 lớp popup (lớp 1 nhấn "Xác nhận"). ⚠ Demo ghi "Người gửi xác nhận đã nhận lại hàng" / "Đơn đóng · hàng đã về người gửi" — khác PRD §8.12.4; STG lệch ⇒ log bug. ✅ QC chốt 2026-09-23: giữ nguyên Expected hiện tại (theo PRD) — không chờ BA. Demo chưa có UI nhóm trạng thái đóng (gộp vào "Hoàn thành", không có "Xem lý do"/"Đăng lại") ⇒ STG giống demo = FAIL + log bug.</t>
         </is>
       </c>
       <c r="N51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
test(vibe): add round 2 retest runs VR-023..VR-028 [AI]
Retest bug In review VR-023..027 (ORD/HOME/CNL/DLV) va VR-028 GIFT:
TC-GIFT-008 PASS. Dong bo Status TC-GIFT-008 vao TC-MASTER v1.1/LATEST,
cap nhat coverage-GIFT, PROGRESS-v1.1 va INDEX.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_test-cases/TC-MASTER-LATEST.xlsx
+++ b/03_test-cases/TC-MASTER-LATEST.xlsx
@@ -20340,7 +20340,11 @@
           <t>Tài khoản 0 đơn/0 quà (test_data_catalog §GIFT v1.1, biên)</t>
         </is>
       </c>
-      <c r="L100" s="5" t="n"/>
+      <c r="L100" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M100" s="5" t="inlineStr">
         <is>
           <t>Mục đích: hết `[GAP]` của `C-ORD-06` phần GIFT (`EMP-08`) — Resolved bằng tài liệu phê duyệt, không còn dựa suy diễn `KB-GIFT-03` như v1.0. · Căn cứ: `DOC-v1.1-01 §8.17.1 EMP-08` · `§6.2 AC-26.2.01`. ⚠️ Cột CTA của `EMP-08` = "—" là assert thật theo `BR17-01` (tối đa 1 CTA) — không phải thiếu sót. · Đã sửa theo delta v1.1 (2026-09-15): đổi Expected từ "KHÔNG hiển thị loại quà nào" (v1.0, suy diễn) sang assert verbatim text + thống kê 0/0 + không CTA (theo tài liệu chính thức).</t>
@@ -39415,7 +39419,11 @@
           <t>Tài khoản 0 đơn/0 quà (test_data_catalog §GIFT v1.1, biên)</t>
         </is>
       </c>
-      <c r="L10" s="5" t="n"/>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Mục đích: hết `[GAP]` của `C-ORD-06` phần GIFT (`EMP-08`) — Resolved bằng tài liệu phê duyệt, không còn dựa suy diễn `KB-GIFT-03` như v1.0. · Căn cứ: `DOC-v1.1-01 §8.17.1 EMP-08` · `§6.2 AC-26.2.01`. ⚠️ Cột CTA của `EMP-08` = "—" là assert thật theo `BR17-01` (tối đa 1 CTA) — không phải thiếu sót. · Đã sửa theo delta v1.1 (2026-09-15): đổi Expected từ "KHÔNG hiển thị loại quà nào" (v1.0, suy diễn) sang assert verbatim text + thống kê 0/0 + không CTA (theo tài liệu chính thức).</t>

</xml_diff>

<commit_message>
docs(ts): apply BA decisions on microsoft forms report [AI]
Theo comment BA tren FE-321..326: mo C-TS-04, sua Then SC-TS-008/009/
012/014 va Expected TC-TS-009/012/013/016/021; TC-TS-017 DESCOPED.
So TC giu nguyen 223 (TS 17).

Refs: N/A
</commit_message>
<xml_diff>
--- a/03_test-cases/TC-MASTER-LATEST.xlsx
+++ b/03_test-cases/TC-MASTER-LATEST.xlsx
@@ -7203,7 +7203,7 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>9. Màn hiển thị "Đã ghi nhận phản hồi" kèm đúng câu "Đội hỗ trợ FoxEco sẽ liên hệ lại số 0912345678 trong vòng 24 giờ làm việc" và nút "Quay lại đơn hàng".</t>
+          <t>9. Màn xác nhận mặc định của Microsoft Forms hiển thị "Đã gửi phản hồi của bạn." (tiếng Anh: "Your response was submitted." — theo ngôn ngữ tài khoản Microsoft), báo cáo được gửi thành công.</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
@@ -7213,12 +7213,12 @@
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: chuỗi cam kết 24 giờ là **thứ duy nhất verify được** của quy trình hỗ trợ — hành động thật của Admin nằm ngoài app, ⛔ không mở rộng phạm vi sang đó. · Căn cứ: `AC-31.1.01` + vibe-check demo 2026-09-15 (ảnh `TS_05`, chuỗi verbatim). Màn xác nhận và nút "Quay lại đơn hàng" do **APP** vẽ chứ không phải trang xác nhận của Google Form (`C-TS-03(d)` Resolved 2026-09-17).</t>
+          <t>🔴 Cập nhật 2026-09-24 theo BA (LinhDCC) trả lời trên Jira `FE-323` (Won't Fix): *"màn hình này là mặc định của Microsoft Form, mình không can thiệp được. Sai tài liệu ạ."* ⇒ Then của `AC-31.1.01` ("Đã ghi nhận phản hồi" + cam kết 24 giờ + nút "Quay lại đơn hàng") là tài liệu sai; ⛔ không assert câu 24 giờ / nút "Quay lại đơn hàng". Kết luận `C-TS-03(d)` (màn do APP vẽ) HẾT HIỆU LỰC — hiện hành `C-TS-04(b)`. · Mục đích: xác nhận luồng gửi hợp lệ đi hết tới màn xác nhận; hành động thật của Admin nằm ngoài app, ⛔ không mở rộng phạm vi.</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
@@ -7458,12 +7458,12 @@
 4. Chọn "Góp ý / đề xuất" ở ô "Loại yêu cầu".
 5. Nhập "App hay bị chậm ở màn bảng tin" vào ô "Mô tả chi tiết".
 6. Nhập "0912abc" vào ô "Số điện thoại liên hệ lại".
-7. Check trạng thái nút "Gửi" cùng phần chữ cạnh nút.</t>
+7. Nhấn "Gửi".&lt;br&gt;8. Check phản hồi của form ở ô "Số điện thoại liên hệ lại" và màn hiện ra sau khi gửi.</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>7. Nút "Gửi" vẫn ở trạng thái bấm được (không disable — cơ chế thật của form là inline error, xem TC-TS-010/TC-TS-011); tuy nhiên SĐT sai định dạng vẫn phải bị chặn không cho gửi (báo lỗi định dạng hoặc tương đương) trước khi form được submit.</t>
+          <t>8. Ô "Số điện thoại liên hệ lại" KHÔNG báo lỗi định dạng; form gửi thành công với giá trị "0912abc" và hiện màn xác nhận mặc định "Đã gửi phản hồi của bạn." (tiếng Anh: "Your response was submitted." — theo ngôn ngữ tài khoản Microsoft) của Microsoft Forms.</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -7473,12 +7473,12 @@
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: nhánh khác bản chất với 2 TC kia — ô CÓ dữ liệu nhưng sai định dạng, dễ bị lập trình thành "chỉ kiểm rỗng". · Căn cứ: `DOC-v1.1-01` §6.2 AC-31.1.02 + §8.16.2. Dùng loại yêu cầu thứ ba để đồng thời phủ đủ 3 giá trị enum của ô "Loại yêu cầu" trong cụm này.</t>
+          <t>🔴 Cập nhật 2026-09-24 theo BA (LinhDCC) trả lời trên Jira `FE-324` (Won't Fix): *"Microsoft form không hỗ trợ rang buộc định dạng số điện thoại -&gt; chấp nhận rủi ro data"* ⇒ nhánh "SĐT không hợp lệ" của `AC-31.1.02` bị bỏ, form chỉ kiểm không rỗng (`C-TS-04(c)`). ⚠️ Test Title còn ghi "vô hiệu hoá khi SĐT sai định dạng" — giữ nguyên vì §10.5 không cho sửa Title; Expected mới là oracle. · Mục đích: chốt rủi ro data đã được BA chấp nhận — nếu form bắt đầu chặn SĐT sai thì cũng là thay đổi cần báo lại.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -7556,7 +7556,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>8. Màn hiển thị "Đã ghi nhận phản hồi", gửi thành công không có thông báo lỗi đòi ảnh.</t>
+          <t>8. Gửi thành công, hiện màn xác nhận mặc định của Microsoft Forms "Đã gửi phản hồi của bạn." (tiếng Anh: "Your response was submitted." — theo ngôn ngữ tài khoản Microsoft), không có thông báo lỗi đòi ảnh.</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -7566,7 +7566,7 @@
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M10" s="6" t="inlineStr">
@@ -7818,7 +7818,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>6. Màn hiển thị thông báo lỗi không tải được kèm nút "Thử lại"; form Google không hiện ra.</t>
+          <t>6. App hiển thị màn lỗi "Không tải được trang" kèm dòng "Vui lòng kiểm tra kết nối mạng và thử lại." và nút "Thử lại"; form Microsoft Forms không hiện ra.</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -7828,12 +7828,12 @@
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §6.2 AC-31.2.01 + **Dev trả lời `C-TS-03(c)` 2026-09-17** (*"App hiển thị nhé"*) — nút "Thử lại" do CHÍNH APP vẽ, tách biệt khỏi khung nhúng, nên assert được dù `BR16-01` dùng Custom Tabs. ⛔ Không assert công nghệ nhúng cụ thể (WebView trần hay Custom Tabs) — không quan sát được từ UI.</t>
+          <t>🔴 Cập nhật lần 2 ngày 2026-09-24 — QC GiangDC2 chốt Expected theo hành vi hiện tại của app (VR-029): mất mạng thì APP tự vẽ màn lỗi + nút "Thử lại", đúng spec gốc `DOC-v1.1-01` §6.2 AC-31.2.01. Bản Expected sửa sáng cùng ngày ("trang lỗi mặc định của WebView, không có nút Thử lại") HẾT HIỆU LỰC — viết khi app còn hiện trang lỗi Chromium `net::ERR_INTERNET_DISCONNECTED` (VR-019, `FE-322` Won't Fix). Status Pass theo evidence `VR-029-TS-2026-09-24/screenshots/TC-TS-016__verify-mat-mang-man-loi-app.png`. Xem `C-TS-04(a)`.</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -7914,12 +7914,12 @@
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="M15" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: fail độc lập với `TC-TS-016` — hiện được nút "Thử lại" không đảm bảo app còn giữ ngữ cảnh đơn; lỗi hay gặp là thử lại xong mở form trắng, mất mã đơn. · Căn cứ: `DOC-v1.1-01` §6.2 AC-31.2.01 (*"KHÔNG mất ngữ cảnh đơn"*).</t>
+          <t>⛔ DESCOPED 2026-09-24 — BA (LinhDCC) trả lời `FE-322` (Won't Fix): *"Form đang dùng là của bên thứ 3 nên mình không kiểm soát được các vấn đề này -&gt; tài liệu sai, bỏ giúp em BR16-04"*. Không còn nút "Thử lại" nên không còn luồng thử lại để kiểm giữ ngữ cảnh đơn. `SC-TS-012` → DEPRECATED (`C-TS-04(a)`). Giữ nguyên dòng theo `Project_rule §10.5`, không tính vào mẫu số coverage.</t>
         </is>
       </c>
       <c r="N15" s="6" t="inlineStr">
@@ -7929,7 +7929,7 @@
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>DESCOPED</t>
         </is>
       </c>
       <c r="P15" s="6" t="inlineStr"/>
@@ -8166,7 +8166,7 @@
 3. Nhấn "Báo cáo sự cố".
 4. Chọn "Sự cố đơn hàng", nhập mô tả "Thử ảnh hưởng trạng thái" và nhập số điện thoại "0912345678".
 5. Nhấn "Gửi".
-6. Nhấn "Quay lại đơn hàng".
+6. Nhấn nút "←" trên thanh tiêu đề để thoát màn xác nhận của Microsoft Forms.
 7. Check trạng thái đơn và nhãn trên màn "Theo dõi đơn".</t>
         </is>
       </c>
@@ -8187,7 +8187,7 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-TS-02(b)` Resolved 2026-09-17 — BA: *"ver hiện tại không chuyển trạng thái gì"*. `§8.12.2` định nghĩa `INCIDENT` = *"có báo cáo sự cố sau khi đơn đã sang IN_TRANSIT"*, đọc được là **tự chuyển**, nên TC này là oracle chặn đúng cách đọc sai đó. · Căn cứ: form Google không gọi được API app ⇒ `INCIDENT` chỉ vào được qua Dev xử lý tay; đơn tự đổi trạng thái ⇒ FAIL và dẫn `C-TS-02`. Kết luận này là căn cứ để `SC-CNL-015`/`SC-DLV-034` out of scope test qua UI.</t>
+          <t>🔴 Cập nhật 2026-09-24 theo BA (LinhDCC) trả lời trên Jira `FE-323`: màn xác nhận là mặc định Microsoft Forms, không có nút "Quay lại đơn hàng" ⇒ step 6 thoát bằng nút "←" của thanh tiêu đề. Mục đích: neo vào `C-TS-02(b)` Resolved 2026-09-17 — BA: *"ver hiện tại không chuyển trạng thái gì"*. `§8.12.2` định nghĩa `INCIDENT` = *"có báo cáo sự cố sau khi đơn đã sang IN_TRANSIT"*, đọc được là **tự chuyển**, nên TC này là oracle chặn đúng cách đọc sai đó. · Căn cứ: form Microsoft Forms không gọi được API app ⇒ `INCIDENT` chỉ vào được qua Dev xử lý tay; đơn tự đổi trạng thái ⇒ FAIL và dẫn `C-TS-02`. Kết luận này là căn cứ để `SC-CNL-015`/`SC-DLV-034` out of scope test qua UI.</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
@@ -8262,22 +8262,22 @@
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>5. Ô "Mã đơn hàng" hiển thị dạng nhãn tĩnh chứ không phải textbox, bàn phím không bật lên, và giá trị trong ô giữ nguyên mã đơn gốc không có ký tự "X".</t>
+          <t>5. Ô "Mã đơn hàng" là ô nhập liệu sửa được: bàn phím bật lên và ký tự "X" được chèn vào giá trị đã điền sẵn.</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>Mã đơn prefill chỉ đọc (test_data_catalog §TS — Mã đơn hàng prefill)</t>
+          <t>Mã đơn prefill — sửa được (test_data_catalog §TS — Mã đơn hàng prefill)</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M22" s="6" t="inlineStr">
         <is>
-          <t>🔴 Áp bản Resolved `C-TS-03(b)` 2026-09-17 — **ĐẢO HẲN Then của `SC-TS-014`** (*"trường prefill CHO PHÉP sửa"*). `§8.16.2` (*"Chỉ đọc · Không sửa"*) là bản đúng, **`BR16-03` là PRD sai**; demo cho thấy ô là nhãn tĩnh, không phải câu trả lời ngắn của Google Form. · Mục đích: kết quả phản trực giác — người chạy đọc `BR16-03` sẽ tưởng "không sửa được" là bug. Sửa được ⇒ FAIL và dẫn `C-TS-03` để BA cập nhật PRD.</t>
+          <t>🔴 Cập nhật 2026-09-24 theo BA (LinhDCC) trả lời trên Jira `FE-326` (Won't Fix): *"Microsoft form không cho phép khoá trường như mô tả → sai tài liệu"* ⇒ `§8.16.2` ("Chỉ đọc · Không sửa") sai tài liệu, `BR16-03` ("người dùng vẫn sửa được") đúng. Kết luận `C-TS-03(b)` (nhãn tĩnh) HẾT HIỆU LỰC — hiện hành `C-TS-04(d)`; Then gốc của `SC-TS-014` có hiệu lực trở lại. ⚠️ Test Title còn ghi "chỉ đọc không sửa được" — giữ nguyên vì §10.5 không cho sửa Title; Expected mới là oracle. Rủi ro đổi nhầm mã đơn được xử lý bằng đối chiếu ở khâu xử lý (`BR16-03`).</t>
         </is>
       </c>
       <c r="N22" s="6" t="inlineStr">
@@ -12013,6 +12013,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
@@ -26131,7 +26132,7 @@
       </c>
       <c r="J171" s="7" t="inlineStr">
         <is>
-          <t>9. Màn hiển thị "Đã ghi nhận phản hồi" kèm đúng câu "Đội hỗ trợ FoxEco sẽ liên hệ lại số 0912345678 trong vòng 24 giờ làm việc" và nút "Quay lại đơn hàng".</t>
+          <t>9. Màn xác nhận mặc định của Microsoft Forms hiển thị "Đã gửi phản hồi của bạn." (tiếng Anh: "Your response was submitted." — theo ngôn ngữ tài khoản Microsoft), báo cáo được gửi thành công.</t>
         </is>
       </c>
       <c r="K171" s="6" t="inlineStr">
@@ -26141,12 +26142,12 @@
       </c>
       <c r="L171" s="6" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M171" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: chuỗi cam kết 24 giờ là **thứ duy nhất verify được** của quy trình hỗ trợ — hành động thật của Admin nằm ngoài app, ⛔ không mở rộng phạm vi sang đó. · Căn cứ: `AC-31.1.01` + vibe-check demo 2026-09-15 (ảnh `TS_05`, chuỗi verbatim). Màn xác nhận và nút "Quay lại đơn hàng" do **APP** vẽ chứ không phải trang xác nhận của Google Form (`C-TS-03(d)` Resolved 2026-09-17).</t>
+          <t>🔴 Cập nhật 2026-09-24 theo BA (LinhDCC) trả lời trên Jira `FE-323` (Won't Fix): *"màn hình này là mặc định của Microsoft Form, mình không can thiệp được. Sai tài liệu ạ."* ⇒ Then của `AC-31.1.01` ("Đã ghi nhận phản hồi" + cam kết 24 giờ + nút "Quay lại đơn hàng") là tài liệu sai; ⛔ không assert câu 24 giờ / nút "Quay lại đơn hàng". Kết luận `C-TS-03(d)` (màn do APP vẽ) HẾT HIỆU LỰC — hiện hành `C-TS-04(b)`. · Mục đích: xác nhận luồng gửi hợp lệ đi hết tới màn xác nhận; hành động thật của Admin nằm ngoài app, ⛔ không mở rộng phạm vi.</t>
         </is>
       </c>
       <c r="N171" s="6" t="inlineStr">
@@ -26379,12 +26380,12 @@
 4. Chọn "Góp ý / đề xuất" ở ô "Loại yêu cầu".
 5. Nhập "App hay bị chậm ở màn bảng tin" vào ô "Mô tả chi tiết".
 6. Nhập "0912abc" vào ô "Số điện thoại liên hệ lại".
-7. Check trạng thái nút "Gửi" cùng phần chữ cạnh nút.</t>
+7. Nhấn "Gửi".&lt;br&gt;8. Check phản hồi của form ở ô "Số điện thoại liên hệ lại" và màn hiện ra sau khi gửi.</t>
         </is>
       </c>
       <c r="J174" s="2" t="inlineStr">
         <is>
-          <t>7. Nút "Gửi" vẫn ở trạng thái bấm được (không disable — cơ chế thật của form là inline error, xem TC-TS-010/TC-TS-011); tuy nhiên SĐT sai định dạng vẫn phải bị chặn không cho gửi (báo lỗi định dạng hoặc tương đương) trước khi form được submit.</t>
+          <t>8. Ô "Số điện thoại liên hệ lại" KHÔNG báo lỗi định dạng; form gửi thành công với giá trị "0912abc" và hiện màn xác nhận mặc định "Đã gửi phản hồi của bạn." (tiếng Anh: "Your response was submitted." — theo ngôn ngữ tài khoản Microsoft) của Microsoft Forms.</t>
         </is>
       </c>
       <c r="K174" s="5" t="inlineStr">
@@ -26394,12 +26395,12 @@
       </c>
       <c r="L174" s="5" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M174" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: nhánh khác bản chất với 2 TC kia — ô CÓ dữ liệu nhưng sai định dạng, dễ bị lập trình thành "chỉ kiểm rỗng". · Căn cứ: `DOC-v1.1-01` §6.2 AC-31.1.02 + §8.16.2. Dùng loại yêu cầu thứ ba để đồng thời phủ đủ 3 giá trị enum của ô "Loại yêu cầu" trong cụm này.</t>
+          <t>🔴 Cập nhật 2026-09-24 theo BA (LinhDCC) trả lời trên Jira `FE-324` (Won't Fix): *"Microsoft form không hỗ trợ rang buộc định dạng số điện thoại -&gt; chấp nhận rủi ro data"* ⇒ nhánh "SĐT không hợp lệ" của `AC-31.1.02` bị bỏ, form chỉ kiểm không rỗng (`C-TS-04(c)`). ⚠️ Test Title còn ghi "vô hiệu hoá khi SĐT sai định dạng" — giữ nguyên vì §10.5 không cho sửa Title; Expected mới là oracle. · Mục đích: chốt rủi ro data đã được BA chấp nhận — nếu form bắt đầu chặn SĐT sai thì cũng là thay đổi cần báo lại.</t>
         </is>
       </c>
       <c r="N174" s="5" t="inlineStr">
@@ -26469,7 +26470,7 @@
       </c>
       <c r="J175" s="7" t="inlineStr">
         <is>
-          <t>6. Màn hiển thị thông báo lỗi không tải được kèm nút "Thử lại"; form Google không hiện ra.</t>
+          <t>6. App hiển thị màn lỗi "Không tải được trang" kèm dòng "Vui lòng kiểm tra kết nối mạng và thử lại." và nút "Thử lại"; form Microsoft Forms không hiện ra.</t>
         </is>
       </c>
       <c r="K175" s="6" t="inlineStr">
@@ -26479,12 +26480,12 @@
       </c>
       <c r="L175" s="6" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M175" s="6" t="inlineStr">
         <is>
-          <t>Căn cứ: `DOC-v1.1-01` §6.2 AC-31.2.01 + **Dev trả lời `C-TS-03(c)` 2026-09-17** (*"App hiển thị nhé"*) — nút "Thử lại" do CHÍNH APP vẽ, tách biệt khỏi khung nhúng, nên assert được dù `BR16-01` dùng Custom Tabs. ⛔ Không assert công nghệ nhúng cụ thể (WebView trần hay Custom Tabs) — không quan sát được từ UI.</t>
+          <t>🔴 Cập nhật lần 2 ngày 2026-09-24 — QC GiangDC2 chốt Expected theo hành vi hiện tại của app (VR-029): mất mạng thì APP tự vẽ màn lỗi + nút "Thử lại", đúng spec gốc `DOC-v1.1-01` §6.2 AC-31.2.01. Bản Expected sửa sáng cùng ngày ("trang lỗi mặc định của WebView, không có nút Thử lại") HẾT HIỆU LỰC — viết khi app còn hiện trang lỗi Chromium `net::ERR_INTERNET_DISCONNECTED` (VR-019, `FE-322` Won't Fix). Status Pass theo evidence `VR-029-TS-2026-09-24/screenshots/TC-TS-016__verify-mat-mang-man-loi-app.png`. Xem `C-TS-04(a)`.</t>
         </is>
       </c>
       <c r="N175" s="6" t="inlineStr">
@@ -26565,12 +26566,12 @@
       </c>
       <c r="L176" s="5" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Skipped</t>
         </is>
       </c>
       <c r="M176" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: fail độc lập với `TC-TS-016` — hiện được nút "Thử lại" không đảm bảo app còn giữ ngữ cảnh đơn; lỗi hay gặp là thử lại xong mở form trắng, mất mã đơn. · Căn cứ: `DOC-v1.1-01` §6.2 AC-31.2.01 (*"KHÔNG mất ngữ cảnh đơn"*).</t>
+          <t>⛔ DESCOPED 2026-09-24 — BA (LinhDCC) trả lời `FE-322` (Won't Fix): *"Form đang dùng là của bên thứ 3 nên mình không kiểm soát được các vấn đề này -&gt; tài liệu sai, bỏ giúp em BR16-04"*. Không còn nút "Thử lại" nên không còn luồng thử lại để kiểm giữ ngữ cảnh đơn. `SC-TS-012` → DEPRECATED (`C-TS-04(a)`). Giữ nguyên dòng theo `Project_rule §10.5`, không tính vào mẫu số coverage.</t>
         </is>
       </c>
       <c r="N176" s="5" t="inlineStr">
@@ -26580,7 +26581,7 @@
       </c>
       <c r="O176" s="5" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>DESCOPED</t>
         </is>
       </c>
       <c r="P176" s="5" t="inlineStr"/>
@@ -26634,7 +26635,7 @@
 3. Nhấn "Báo cáo sự cố".
 4. Chọn "Sự cố đơn hàng", nhập mô tả "Thử ảnh hưởng trạng thái" và nhập số điện thoại "0912345678".
 5. Nhấn "Gửi".
-6. Nhấn "Quay lại đơn hàng".
+6. Nhấn nút "←" trên thanh tiêu đề để thoát màn xác nhận của Microsoft Forms.
 7. Check trạng thái đơn và nhãn trên màn "Theo dõi đơn".</t>
         </is>
       </c>
@@ -26655,7 +26656,7 @@
       </c>
       <c r="M177" s="6" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-TS-02(b)` Resolved 2026-09-17 — BA: *"ver hiện tại không chuyển trạng thái gì"*. `§8.12.2` định nghĩa `INCIDENT` = *"có báo cáo sự cố sau khi đơn đã sang IN_TRANSIT"*, đọc được là **tự chuyển**, nên TC này là oracle chặn đúng cách đọc sai đó. · Căn cứ: form Google không gọi được API app ⇒ `INCIDENT` chỉ vào được qua Dev xử lý tay; đơn tự đổi trạng thái ⇒ FAIL và dẫn `C-TS-02`. Kết luận này là căn cứ để `SC-CNL-015`/`SC-DLV-034` out of scope test qua UI.</t>
+          <t>🔴 Cập nhật 2026-09-24 theo BA (LinhDCC) trả lời trên Jira `FE-323`: màn xác nhận là mặc định Microsoft Forms, không có nút "Quay lại đơn hàng" ⇒ step 6 thoát bằng nút "←" của thanh tiêu đề. Mục đích: neo vào `C-TS-02(b)` Resolved 2026-09-17 — BA: *"ver hiện tại không chuyển trạng thái gì"*. `§8.12.2` định nghĩa `INCIDENT` = *"có báo cáo sự cố sau khi đơn đã sang IN_TRANSIT"*, đọc được là **tự chuyển**, nên TC này là oracle chặn đúng cách đọc sai đó. · Căn cứ: form Microsoft Forms không gọi được API app ⇒ `INCIDENT` chỉ vào được qua Dev xử lý tay; đơn tự đổi trạng thái ⇒ FAIL và dẫn `C-TS-02`. Kết luận này là căn cứ để `SC-CNL-015`/`SC-DLV-034` out of scope test qua UI.</t>
         </is>
       </c>
       <c r="N177" s="6" t="inlineStr">
@@ -26977,7 +26978,7 @@
       </c>
       <c r="J181" s="7" t="inlineStr">
         <is>
-          <t>8. Màn hiển thị "Đã ghi nhận phản hồi", gửi thành công không có thông báo lỗi đòi ảnh.</t>
+          <t>8. Gửi thành công, hiện màn xác nhận mặc định của Microsoft Forms "Đã gửi phản hồi của bạn." (tiếng Anh: "Your response was submitted." — theo ngôn ngữ tài khoản Microsoft), không có thông báo lỗi đòi ảnh.</t>
         </is>
       </c>
       <c r="K181" s="6" t="inlineStr">
@@ -26987,7 +26988,7 @@
       </c>
       <c r="L181" s="6" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M181" s="6" t="inlineStr">
@@ -27399,22 +27400,22 @@
       </c>
       <c r="J186" s="2" t="inlineStr">
         <is>
-          <t>5. Ô "Mã đơn hàng" hiển thị dạng nhãn tĩnh chứ không phải textbox, bàn phím không bật lên, và giá trị trong ô giữ nguyên mã đơn gốc không có ký tự "X".</t>
+          <t>5. Ô "Mã đơn hàng" là ô nhập liệu sửa được: bàn phím bật lên và ký tự "X" được chèn vào giá trị đã điền sẵn.</t>
         </is>
       </c>
       <c r="K186" s="5" t="inlineStr">
         <is>
-          <t>Mã đơn prefill chỉ đọc (test_data_catalog §TS — Mã đơn hàng prefill)</t>
+          <t>Mã đơn prefill — sửa được (test_data_catalog §TS — Mã đơn hàng prefill)</t>
         </is>
       </c>
       <c r="L186" s="5" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="M186" s="5" t="inlineStr">
         <is>
-          <t>🔴 Áp bản Resolved `C-TS-03(b)` 2026-09-17 — **ĐẢO HẲN Then của `SC-TS-014`** (*"trường prefill CHO PHÉP sửa"*). `§8.16.2` (*"Chỉ đọc · Không sửa"*) là bản đúng, **`BR16-03` là PRD sai**; demo cho thấy ô là nhãn tĩnh, không phải câu trả lời ngắn của Google Form. · Mục đích: kết quả phản trực giác — người chạy đọc `BR16-03` sẽ tưởng "không sửa được" là bug. Sửa được ⇒ FAIL và dẫn `C-TS-03` để BA cập nhật PRD.</t>
+          <t>🔴 Cập nhật 2026-09-24 theo BA (LinhDCC) trả lời trên Jira `FE-326` (Won't Fix): *"Microsoft form không cho phép khoá trường như mô tả → sai tài liệu"* ⇒ `§8.16.2` ("Chỉ đọc · Không sửa") sai tài liệu, `BR16-03` ("người dùng vẫn sửa được") đúng. Kết luận `C-TS-03(b)` (nhãn tĩnh) HẾT HIỆU LỰC — hiện hành `C-TS-04(d)`; Then gốc của `SC-TS-014` có hiệu lực trở lại. ⚠️ Test Title còn ghi "chỉ đọc không sửa được" — giữ nguyên vì §10.5 không cho sửa Title; Expected mới là oracle. Rủi ro đổi nhầm mã đơn được xử lý bằng đối chiếu ở khâu xử lý (`BR16-03`).</t>
         </is>
       </c>
       <c r="N186" s="5" t="inlineStr">

</xml_diff>